<commit_message>
Refactor directory structure: rename 'random_posterior_sampling_analysis' to 'SI_11_and_SHAP_analysis' and update associated paths in the README. Remove obsolete files and scripts related to random posterior sampling analysis.
</commit_message>
<xml_diff>
--- a/performence tests/summery_of_error_analysis.xlsx
+++ b/performence tests/summery_of_error_analysis.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/alon/navehr/PerformenceTests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/navehr/Dropbox/naveh/weizmann/uri alon/aging/code_3/ComparativeAgingV3/performence tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{914F98A2-88C8-784F-89AD-FE992B8B7FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD39ED75-E97C-C446-B101-0B54C8FB7C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-9620" yWindow="-28800" windowWidth="51200" windowHeight="28800" xr2:uid="{DB8EA1E4-65D9-DD48-9A84-B30F779C94E6}"/>
+    <workbookView xWindow="-9620" yWindow="-28300" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{DB8EA1E4-65D9-DD48-9A84-B30F779C94E6}"/>
   </bookViews>
   <sheets>
     <sheet name="summery_error_summary" sheetId="1" r:id="rId1"/>
+    <sheet name="README" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">summery_error_summary!$A$1:$Q$621</definedName>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1293" uniqueCount="88">
   <si>
     <t>config</t>
   </si>
@@ -228,12 +229,72 @@
   <si>
     <t>mice_M_weeks_test</t>
   </si>
+  <si>
+    <t>Config names meaning</t>
+  </si>
+  <si>
+    <t>the config name consists of the organism most similar to the parameter set used and the number of individule simulated in each dataset, so celegans1000 would be the results for 5 tests with C elegans like parameters, for each we generated a different simulated dataset with a 1000 individuals</t>
+  </si>
+  <si>
+    <t>The parameter or parameter groups whos statistics are shown</t>
+  </si>
+  <si>
+    <t>The avarge over 5 runs of the error of the mean of the MCMC samples (not used in the paper)</t>
+  </si>
+  <si>
+    <t>The std over 5 runs of the error of the mean of the MCMC samples (not used in the paper)</t>
+  </si>
+  <si>
+    <t>The median over 5 runs of the error of the mean of the MCMC samples (not used in the paper)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The avarge over 5 runs of the error of the mode (highest marginal posterior probability) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The std over 5 runs of the error of the mode (highest marginal posterior probability) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The median over 5 runs of the error of the mode (highest marginal posterior probability) </t>
+  </si>
+  <si>
+    <t>The avarge over 5 runs of the error of the mode mode overall (After binning the MCMC samples (with averaging of likelihoods that fall in the same bin), the mode overall contains the sample with the highest likelihood within the mode bin (the bin with highest posterior probability)</t>
+  </si>
+  <si>
+    <t>The std over 5 runs of the error of the mode mode overall (After binning the MCMC samples (with averaging of likelihoods that fall in the same bin), the mode overall contains the sample with the highest likelihood within the mode bin (the bin with highest posterior probability)</t>
+  </si>
+  <si>
+    <t>The median over 5 runs of the error of the mode mode overall (After binning the MCMC samples (with averaging of likelihoods that fall in the same bin), the mode overall contains the sample with the highest likelihood within the mode bin (the bin with highest posterior probability)</t>
+  </si>
+  <si>
+    <t>GENRAL NOTE</t>
+  </si>
+  <si>
+    <t>all values are presented in % of the truth value. Since intervals and errors may be non symmetric, error or CI can be larger then 100% (for instance an estimate which is 10 times larger then the truth value is a 1000% error)</t>
+  </si>
+  <si>
+    <t>The avarge over 5 runs of the size of the 95%CI (calclulated over the marginalized posterior)</t>
+  </si>
+  <si>
+    <t>The std over 5 runs of the size of the 95%CI (calclulated over the marginalized posterior)</t>
+  </si>
+  <si>
+    <t>The percent out of 5 runs of the truth value falling within the 16%CI (calclulated over the marginalized posterior)</t>
+  </si>
+  <si>
+    <t>The percent out of 5 runs of the truth value falling within the 50%CI (calclulated over the marginalized posterior)</t>
+  </si>
+  <si>
+    <t>The percent out of 5 runs of the truth value falling within the 95%CI (calclulated over the marginalized posterior)</t>
+  </si>
+  <si>
+    <t>The percent out of 5 runs of the truth value falling within the log(mean)+-log(std) interval</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -364,6 +425,20 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -710,8 +785,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1089,6 +1166,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA4A2DC9-8EFE-914B-8454-6AABC8A51EDD}">
   <dimension ref="A1:Q621"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -28367,4 +28461,161 @@
   <autoFilter ref="A1:Q621" xr:uid="{BA4A2DC9-8EFE-914B-8454-6AABC8A51EDD}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C1A353-75CD-0D47-882D-7CB04F8827D5}">
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>